<commit_message>
Final: Clean app with section fix and templates folder
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwwro\attendance_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B705F8-936D-42AE-98F8-5F2256110EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012F86E6-FC5B-46D1-8204-46E94F616AA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F2D1DCF1-8ADF-42F5-8EEB-A3EBD4A5ED5A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="22">
   <si>
     <t>student_id</t>
   </si>
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1CB3C71-5FD0-48F1-A7C3-9F21CDE528D9}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
@@ -652,6 +652,686 @@
         <v>12345</v>
       </c>
     </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>111</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12">
+        <v>2331223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>112</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13">
+        <v>56678</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>113</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14">
+        <v>345567</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>114</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <v>56778</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>115</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16">
+        <v>55667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>116</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17">
+        <v>67899</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>117</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>23454</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>118</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>119</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20">
+        <v>23678</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>120</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>121</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22">
+        <v>2331223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>122</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23">
+        <v>56678</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>123</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24">
+        <v>345567</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>124</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25">
+        <v>56778</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>125</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26">
+        <v>55667</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>126</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27">
+        <v>67899</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>127</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28">
+        <v>23454</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>128</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>129</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30">
+        <v>23678</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>130</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>131</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32">
+        <v>2331223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>132</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33">
+        <v>56678</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>133</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34">
+        <v>345567</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="2">
+        <v>134</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35">
+        <v>56778</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="2">
+        <v>135</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E36">
+        <v>55667</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2">
+        <v>136</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37">
+        <v>67899</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2">
+        <v>137</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>23454</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2">
+        <v>138</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2">
+        <v>139</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E40">
+        <v>23678</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2">
+        <v>140</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E41">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2">
+        <v>141</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E42">
+        <v>2331223</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2">
+        <v>142</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43">
+        <v>56678</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2">
+        <v>143</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E44">
+        <v>345567</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2">
+        <v>144</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E45">
+        <v>56778</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2">
+        <v>145</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E46">
+        <v>55667</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2">
+        <v>146</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>67899</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2">
+        <v>147</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48">
+        <v>23454</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2">
+        <v>148</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E49">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2">
+        <v>149</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50">
+        <v>23678</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2">
+        <v>150</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E51">
+        <v>12345</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>